<commit_message>
Rendre les cases de saisie lisibles en mode sombre (texte gris foncé, fond plus clair)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNt8QQ6oyZWdcVMAnmdvTM
</commit_message>
<xml_diff>
--- a/produit-budget-famille/Budget-Famille-Sans-Stress.xlsx
+++ b/produit-budget-famille/Budget-Famille-Sans-Stress.xlsx
@@ -352,7 +352,7 @@
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="168" formatCode="0%;\-0%;\-"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -377,7 +377,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="18"/>
+      <sz val="16"/>
       <color rgb="FF2E7D6B"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -415,13 +415,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
@@ -440,7 +433,7 @@
     <font>
       <i val="true"/>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF555555"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -485,12 +478,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFE3F2EE"/>
+        <bgColor rgb="FFFFF7D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF4C2"/>
+        <fgColor rgb="FFFFF7D6"/>
         <bgColor rgb="FFFFE8CC"/>
       </patternFill>
     </fill>
@@ -589,19 +582,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -609,7 +602,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -617,35 +610,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -665,7 +658,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -732,7 +725,7 @@
       <rgbColor rgb="FF7A9346"/>
       <rgbColor rgb="FF7E9BC7"/>
       <rgbColor rgb="FF973F3C"/>
-      <rgbColor rgb="FFFFF4C2"/>
+      <rgbColor rgb="FFFFF7D6"/>
       <rgbColor rgb="FFE3F2EE"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFE78C41"/>
@@ -765,7 +758,7 @@
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF2E7D6B"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF555555"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FFB34A48"/>
       <rgbColor rgb="FF654E7F"/>
@@ -1664,13 +1657,13 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>101160</xdr:rowOff>
+      <xdr:rowOff>131040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>147600</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>81360</xdr:rowOff>
+      <xdr:rowOff>111240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3010,7 +3003,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
@@ -4266,7 +4259,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>47</v>
       </c>
@@ -9992,7 +9985,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>59</v>
       </c>
@@ -11471,7 +11464,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>70</v>
       </c>

</xml_diff>